<commit_message>
aligning rc and wb
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25_12_11.xlsx
+++ b/simulations/scene/inputs/Scenarios_25_12_11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp54510\work_home\tigerault\Wheat-BRIDGES_framework\Root-CyNAPS\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1762FF8-D615-4F88-A1F7-2E488AC900AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD979268-BC1C-4272-97D7-F893FA96465F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -4191,43 +4191,43 @@
         <v>0.1</v>
       </c>
       <c r="H35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="I35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="J35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="K35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="L35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="M35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="N35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="O35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="P35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="Q35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="R35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="S35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="T35" s="10">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
@@ -4560,17 +4560,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:T8">
+    <cfRule type="colorScale" priority="764">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="763">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="764">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4582,17 +4582,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:T9">
+    <cfRule type="colorScale" priority="766">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="765">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="766">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4648,17 +4648,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13:T13">
+    <cfRule type="colorScale" priority="772">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="771">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="772">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4670,17 +4670,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14:T14">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4692,17 +4692,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15:T15">
+    <cfRule type="colorScale" priority="62">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="61">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="62">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4758,17 +4758,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H19:T19">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="46">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4868,17 +4868,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24:T27">
+    <cfRule type="colorScale" priority="780">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="779">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="780">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4890,17 +4890,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28:T28">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4934,17 +4934,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30:T31">
+    <cfRule type="colorScale" priority="755">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="754">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="755">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4966,6 +4966,16 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="min"/>
@@ -4977,16 +4987,6 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5040,17 +5040,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H34:T34">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5084,17 +5084,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
+    <cfRule type="colorScale" priority="182">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="181">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="182">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5162,17 +5162,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3">
+    <cfRule type="colorScale" priority="180">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="179">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="180">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5184,17 +5184,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3">
+    <cfRule type="colorScale" priority="178">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="177">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="178">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5206,17 +5206,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3">
+    <cfRule type="colorScale" priority="176">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="175">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="176">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5228,17 +5228,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3">
+    <cfRule type="colorScale" priority="174">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="173">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="174">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5250,17 +5250,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N3">
+    <cfRule type="colorScale" priority="172">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="171">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="172">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5272,17 +5272,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O3">
+    <cfRule type="colorScale" priority="170">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="169">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="170">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5316,17 +5316,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3">
+    <cfRule type="colorScale" priority="166">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="165">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="166">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5382,17 +5382,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T3">
+    <cfRule type="colorScale" priority="158">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="157">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="158">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>